<commit_message>
Update reports 2026-09-29 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-29.xlsx
+++ b/gex_pivot_levels_2026-09-29.xlsx
@@ -610,12 +610,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$18.62M</t>
+          <t>-$17.00M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$19.43M</t>
+          <t>+$17.74M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -643,12 +643,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>-$2.12M</t>
+          <t>-$1.96M</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$2.51M</t>
+          <t>+$2.32M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -734,12 +734,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$26.11M</t>
+          <t>-$26.53M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$39.00M</t>
+          <t>+$39.63M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -767,12 +767,12 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>+$1.91M</t>
+          <t>+$1.94M</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>+$8.91M</t>
+          <t>+$9.04M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>-$20.85M</t>
+          <t>-$21.43M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+$35.59M</t>
+          <t>+$36.59M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>-$415.84K</t>
+          <t>-$431.06K</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>+$24.50M</t>
+          <t>+$25.39M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>+$599.48K</t>
+          <t>+$621.15K</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>+$42.14M</t>
+          <t>+$43.67M</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$12.26M</t>
+          <t>+$12.44M</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>+$23.23M</t>
+          <t>+$23.58M</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>+$14.67M</t>
+          <t>+$14.91M</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>+$18.48M</t>
+          <t>+$18.79M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -3044,12 +3044,12 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>+$599.48K</t>
+          <t>+$621.15K</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>+$42.14M</t>
+          <t>+$43.67M</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3078,12 +3078,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>-$26.11M</t>
+          <t>-$26.53M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+$39.00M</t>
+          <t>+$39.63M</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3116,12 +3116,12 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>-$20.85M</t>
+          <t>-$21.43M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$35.59M</t>
+          <t>+$36.59M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3180,24 +3180,24 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>7720.13</v>
+        <v>7717.56</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>765</v>
+        <v>7675</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>-$11.25M</t>
+          <t>-$431.06K</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>+$24.75M</t>
+          <t>+$25.39M</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3214,24 +3214,24 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>7717.56</v>
+        <v>7720.13</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>7675</v>
+        <v>765</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>-$415.84K</t>
+          <t>-$11.25M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>+$24.50M</t>
+          <t>+$24.75M</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -3260,12 +3260,12 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>+$12.26M</t>
+          <t>+$12.44M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>+$23.23M</t>
+          <t>+$23.58M</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -3352,78 +3352,78 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="5" t="n">
+        <v>7767.56</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>7725</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>+$14.91M</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>+$18.79M</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
         <v>7642.56</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C14" s="2" t="n">
         <v>7600</v>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>-$18.62M</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>+$19.43M</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>-$17.00M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>+$17.74M</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>7767.56</v>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>7725</v>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>+$14.67M</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>+$18.48M</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3590,12 +3590,12 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>+$1.91M</t>
+          <t>+$1.94M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>+$8.91M</t>
+          <t>+$9.04M</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -4068,12 +4068,12 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>-$2.12M</t>
+          <t>-$1.96M</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>+$2.51M</t>
+          <t>+$2.32M</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">

</xml_diff>